<commit_message>
Publish catalog from admin
</commit_message>
<xml_diff>
--- a/data/Euro_Coin_Catalog_Automation.xlsx
+++ b/data/Euro_Coin_Catalog_Automation.xlsx
@@ -1320,23 +1320,81 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="6" t="n"/>
-      <c r="J12" s="7" t="n"/>
-      <c r="K12" s="5" t="n"/>
-      <c r="L12" s="6" t="n"/>
-      <c r="M12" s="5" t="n"/>
-      <c r="N12" s="5" t="n"/>
-      <c r="O12" s="5" t="n"/>
-      <c r="P12" s="8" t="n"/>
-      <c r="Q12" s="6" t="n"/>
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>013</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>1 €</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>1 Euro</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>Collection</t>
+        </is>
+      </c>
+      <c r="J12" s="14" t="inlineStr"/>
+      <c r="K12" s="12" t="inlineStr">
+        <is>
+          <t>013_Belgium_2002_1Euro_Regular.jpeg</t>
+        </is>
+      </c>
+      <c r="L12" s="13" t="inlineStr"/>
+      <c r="M12" s="12" t="inlineStr">
+        <is>
+          <t>Bimetallic</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr">
+        <is>
+          <t>7.50 g</t>
+        </is>
+      </c>
+      <c r="O12" s="12" t="inlineStr">
+        <is>
+          <t>23.25 mm</t>
+        </is>
+      </c>
+      <c r="P12" s="15" t="inlineStr">
+        <is>
+          <t>Regular 1 € circulation coin of Belgium.</t>
+        </is>
+      </c>
+      <c r="Q12" s="16" t="inlineStr">
+        <is>
+          <t>The first series depicts King Albert II in the inner part of the coin, while the royal monogram - a capital "A" underneath a crown - among 12 stars, symbolising Europe, as well as the year of issuance appear in the outer part.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="5" t="n"/>

</xml_diff>